<commit_message>
update output data (first assessment)
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output_base_test.xlsx
+++ b/00_code_base/02_unidirectional/output_base_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\00_code_base\02_unidirectional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4702AEC-6750-4AFB-9092-40CC660B7F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1ADB1B3-50B3-440D-BF7F-5CE0A52BE5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw" sheetId="1" r:id="rId1"/>
@@ -1307,6 +1307,13 @@
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
+      <border outline="0">
+        <bottom style="thick">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1341,13 +1348,6 @@
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thick">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
@@ -1358,34 +1358,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -1421,6 +1393,34 @@
         <horizontal/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1435,196 +1435,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F8C1A0C6-C4C4-4C45-B104-B3FE75F0BAEF}" name="Table1" displayName="Table1" ref="A1:E372" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:E372" xr:uid="{F8C1A0C6-C4C4-4C45-B104-B3FE75F0BAEF}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="AF', 'AF_LNG_exp'"/>
-        <filter val="AF_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="AF_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="AU', 'AU_LNG_exp'"/>
-        <filter val="AU_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="AU_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="EG', 'EG_LNG_exp'"/>
-        <filter val="EG_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="EG_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="IM', 'IM_LNG_exp'"/>
-        <filter val="IM_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="IM_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="ME', 'ME_LNG_exp'"/>
-        <filter val="ME_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="ME_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="QA', 'QA_LNG_exp'"/>
-        <filter val="QA_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="QA_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="RU', 'RU_LNG_exp'"/>
-        <filter val="RU_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="RU_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="TT', 'TT_LNG_exp'"/>
-        <filter val="TT_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="TT_LNG_exp', 'UK_LNG_imp'"/>
-        <filter val="USA', 'USA_LNG_exp'"/>
-        <filter val="USA_LNG_exp', 'AF_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'AS_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'BE_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'CN_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'EG_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'EL_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'ES_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'FR_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'HR_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'IN_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'IT_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'JS_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'LT_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'NL_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'PL_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'PT_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'SA_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'TR_LNG_imp'"/>
-        <filter val="USA_LNG_exp', 'UK_LNG_imp'"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F8C1A0C6-C4C4-4C45-B104-B3FE75F0BAEF}" name="Table1" displayName="Table1" ref="A1:E372" totalsRowShown="0" headerRowDxfId="9">
+  <autoFilter ref="A1:E372" xr:uid="{F8C1A0C6-C4C4-4C45-B104-B3FE75F0BAEF}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E372">
     <sortCondition ref="C1:C372"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{EDC06B4A-496B-4E5E-ADDB-C8366DA2F7CA}" name="Column1" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{EDC06B4A-496B-4E5E-ADDB-C8366DA2F7CA}" name="Column1" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{CCDC4B9D-ABBF-404F-B073-562B735615DA}" name="Commodity"/>
     <tableColumn id="3" xr3:uid="{AA66E3A0-18A3-4298-A944-9648AEFDC782}" name="Edge"/>
     <tableColumn id="4" xr3:uid="{2B54A453-DE4A-459E-9A0B-D43757EE9861}" name="Flow (GWh)"/>
@@ -1642,7 +1459,7 @@
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{0E30B145-4D3F-4FAD-BD41-21ABAB04B6EC}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{757D861D-FB27-46FF-B0C9-F12A4872D22A}" name="Flow (GWh)" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{757D861D-FB27-46FF-B0C9-F12A4872D22A}" name="Flow (GWh)" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{B42BA0CA-AAF3-4240-B01E-874DB68E1F64}" name="Share"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1654,10 +1471,10 @@
   <autoFilter ref="A1:C14" xr:uid="{3417075B-B51B-429B-8BA8-43E190BF8519}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{A239A1DC-0210-4956-ABE7-EF6CDA5A30E2}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{322E7DE0-B95E-46AC-9403-C71D0E63B73A}" name="Flow (GWh)" dataDxfId="7">
+    <tableColumn id="2" xr3:uid="{322E7DE0-B95E-46AC-9403-C71D0E63B73A}" name="Flow (GWh)" dataDxfId="6">
       <calculatedColumnFormula>VLOOKUP(LNG_Import_use!$A2,Raw!$C$3:$E$372,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E19B88D8-3893-4610-AB1D-CF00C32B1D5C}" name="Share" dataDxfId="6">
+    <tableColumn id="3" xr3:uid="{E19B88D8-3893-4610-AB1D-CF00C32B1D5C}" name="Share" dataDxfId="5">
       <calculatedColumnFormula>VLOOKUP(LNG_Import_use!$A2,Raw!$C$3:$E$372,3,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1670,7 +1487,7 @@
   <autoFilter ref="A1:B17" xr:uid="{A8372A6F-EB83-42B1-A6B1-D9A865C31E2A}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D3B0A0F4-AE4B-4C05-803A-8265FB2E0BEC}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{3D272239-DFA1-4C23-990B-17340DB0F202}" name="Flow (GWh)" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{3D272239-DFA1-4C23-990B-17340DB0F202}" name="Flow (GWh)" dataDxfId="4">
       <calculatedColumnFormula>SUMIFS(Raw!$D$2:$D$371,Raw!$C$2:$C$371,"*"&amp;LNG_Sources!$A2&amp;"*")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1679,7 +1496,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1122FFF2-C470-41D5-B466-2B2A16A0702F}" name="Table7" displayName="Table7" ref="D1:E6" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{1122FFF2-C470-41D5-B466-2B2A16A0702F}" name="Table7" displayName="Table7" ref="D1:E6" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2">
   <autoFilter ref="D1:E6" xr:uid="{1122FFF2-C470-41D5-B466-2B2A16A0702F}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{4B792274-18C2-4C26-B54A-695915F3118E}" name="Region"/>
@@ -1694,7 +1511,7 @@
   <autoFilter ref="A1:B33" xr:uid="{8121B5DA-0937-487A-A3DF-77ACBB8999F9}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{03B06CF4-5F36-4B7E-8CC9-8D06BB4532D5}" name="Edge"/>
-    <tableColumn id="2" xr3:uid="{1AD1E774-B856-4665-89D5-9C7DC08BC3A8}" name="Flow (GWh)" dataDxfId="5">
+    <tableColumn id="2" xr3:uid="{1AD1E774-B856-4665-89D5-9C7DC08BC3A8}" name="Flow (GWh)" dataDxfId="0">
       <calculatedColumnFormula>VLOOKUP($A2,Raw!$C$3:$E$372,2,FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2336,7 +2153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>126</v>
       </c>
@@ -2353,7 +2170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>361</v>
       </c>
@@ -2370,7 +2187,7 @@
         <v>7.5638907995223673E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>20</v>
       </c>
@@ -2387,7 +2204,7 @@
         <v>0.44863195343807849</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>316</v>
       </c>
@@ -2404,7 +2221,7 @@
         <v>5.5586420558642063E-5</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>144</v>
       </c>
@@ -2421,7 +2238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>121</v>
       </c>
@@ -2438,7 +2255,7 @@
         <v>3.3990227793548183E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>367</v>
       </c>
@@ -2455,7 +2272,7 @@
         <v>0.15143218864165439</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>16</v>
       </c>
@@ -2472,7 +2289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>102</v>
       </c>
@@ -2489,7 +2306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>9</v>
       </c>
@@ -2506,7 +2323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>43</v>
       </c>
@@ -2523,7 +2340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>26</v>
       </c>
@@ -2540,7 +2357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>318</v>
       </c>
@@ -2897,7 +2714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>363</v>
       </c>
@@ -2914,7 +2731,7 @@
         <v>0.1412790259322253</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>321</v>
       </c>
@@ -2931,7 +2748,7 @@
         <v>2.9070907268661822E-4</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>1</v>
       </c>
@@ -2948,7 +2765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>10</v>
       </c>
@@ -2965,7 +2782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>2</v>
       </c>
@@ -2982,7 +2799,7 @@
         <v>0.46077157072013109</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>90</v>
       </c>
@@ -2999,7 +2816,7 @@
         <v>0.58876973703138435</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>18</v>
       </c>
@@ -3016,7 +2833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>110</v>
       </c>
@@ -3033,7 +2850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>320</v>
       </c>
@@ -3050,7 +2867,7 @@
         <v>5.7643005764300594E-6</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>104</v>
       </c>
@@ -3067,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>30</v>
       </c>
@@ -3084,7 +2901,7 @@
         <v>0.31767289927026832</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>53</v>
       </c>
@@ -3101,7 +2918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>45</v>
       </c>
@@ -3118,7 +2935,7 @@
         <v>0.76431262521706622</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>11</v>
       </c>
@@ -3135,7 +2952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>322</v>
       </c>
@@ -3152,7 +2969,7 @@
         <v>5.3100932310093232E-5</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>38</v>
       </c>
@@ -3169,7 +2986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>35</v>
       </c>
@@ -3186,7 +3003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>91</v>
       </c>
@@ -3203,7 +3020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>319</v>
       </c>
@@ -3220,7 +3037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>65</v>
       </c>
@@ -3237,7 +3054,7 @@
         <v>0.43679474381909389</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -3254,7 +3071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>92</v>
       </c>
@@ -3271,7 +3088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>349</v>
       </c>
@@ -3288,7 +3105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>139</v>
       </c>
@@ -3305,7 +3122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>356</v>
       </c>
@@ -3322,7 +3139,7 @@
         <v>0.19651212010048549</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>122</v>
       </c>
@@ -3339,7 +3156,7 @@
         <v>7.6614510084955484E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>364</v>
       </c>
@@ -3356,7 +3173,7 @@
         <v>0.18954702522313899</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>137</v>
       </c>
@@ -3373,7 +3190,7 @@
         <v>0.72749775510554204</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>146</v>
       </c>
@@ -3390,7 +3207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>368</v>
       </c>
@@ -3407,7 +3224,7 @@
         <v>0.16600286255708821</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>12</v>
       </c>
@@ -3424,7 +3241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>106</v>
       </c>
@@ -3441,7 +3258,7 @@
         <v>0.52417236464449013</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>17</v>
       </c>
@@ -3458,7 +3275,7 @@
         <v>6.1267584861917197E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>324</v>
       </c>
@@ -3475,7 +3292,7 @@
         <v>1.9156529415652939E-4</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>25</v>
       </c>
@@ -3492,7 +3309,7 @@
         <v>0.58433262178048562</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>0</v>
       </c>
@@ -3509,7 +3326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>28</v>
       </c>
@@ -3526,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>54</v>
       </c>
@@ -3543,7 +3360,7 @@
         <v>0.17314059731274831</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>87</v>
       </c>
@@ -3560,7 +3377,7 @@
         <v>0.37088610763530178</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>107</v>
       </c>
@@ -3577,7 +3394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>99</v>
       </c>
@@ -3594,7 +3411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>50</v>
       </c>
@@ -3611,7 +3428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>62</v>
       </c>
@@ -3628,7 +3445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>329</v>
       </c>
@@ -3645,7 +3462,7 @@
         <v>4.7618984761898476E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>57</v>
       </c>
@@ -3662,7 +3479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>82</v>
       </c>
@@ -3679,7 +3496,7 @@
         <v>0.64693199131306389</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>325</v>
       </c>
@@ -3696,7 +3513,7 @@
         <v>1.39470769647077E-3</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>84</v>
       </c>
@@ -3713,7 +3530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>19</v>
       </c>
@@ -3730,7 +3547,7 @@
         <v>5.6905849187011401E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>88</v>
       </c>
@@ -3747,7 +3564,7 @@
         <v>0.87862567559067184</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>317</v>
       </c>
@@ -3764,7 +3581,7 @@
         <v>7.9551854367685429E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>59</v>
       </c>
@@ -3781,7 +3598,7 @@
         <v>5.9466984921288171E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>32</v>
       </c>
@@ -3798,7 +3615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>326</v>
       </c>
@@ -4138,7 +3955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="1">
         <v>123</v>
       </c>
@@ -4155,7 +3972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="1">
         <v>369</v>
       </c>
@@ -4172,7 +3989,7 @@
         <v>5.7120480864135487E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="1">
         <v>52</v>
       </c>
@@ -4189,7 +4006,7 @@
         <v>0.4889154838235395</v>
       </c>
     </row>
-    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="1">
         <v>64</v>
       </c>
@@ -4206,7 +4023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="1">
         <v>108</v>
       </c>
@@ -4223,7 +4040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="1">
         <v>330</v>
       </c>
@@ -4240,7 +4057,7 @@
         <v>6.3309606330960652E-6</v>
       </c>
     </row>
-    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="1">
         <v>48</v>
       </c>
@@ -4257,7 +4074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="1">
         <v>79</v>
       </c>
@@ -4274,7 +4091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="1">
         <v>112</v>
       </c>
@@ -4291,7 +4108,7 @@
         <v>0.60845975467145264</v>
       </c>
     </row>
-    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="1">
         <v>354</v>
       </c>
@@ -4308,7 +4125,7 @@
         <v>4.4942004494200447E-5</v>
       </c>
     </row>
-    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
         <v>15</v>
       </c>
@@ -4325,7 +4142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="1">
         <v>327</v>
       </c>
@@ -4342,7 +4159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="1">
         <v>40</v>
       </c>
@@ -4359,7 +4176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="1">
         <v>95</v>
       </c>
@@ -4376,7 +4193,7 @@
         <v>0.73633950725805031</v>
       </c>
     </row>
-    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="1">
         <v>93</v>
       </c>
@@ -4393,7 +4210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="1">
         <v>118</v>
       </c>
@@ -4410,7 +4227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="1">
         <v>328</v>
       </c>
@@ -4427,7 +4244,7 @@
         <v>1.694997469499747E-5</v>
       </c>
     </row>
-    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="1">
         <v>3</v>
       </c>
@@ -4444,7 +4261,7 @@
         <v>0.30397553284426598</v>
       </c>
     </row>
-    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="1">
         <v>5</v>
       </c>
@@ -4461,7 +4278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="1">
         <v>113</v>
       </c>
@@ -4478,7 +4295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="1">
         <v>323</v>
       </c>
@@ -4495,7 +4312,7 @@
         <v>8.6795223179522317E-4</v>
       </c>
     </row>
-    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="1">
         <v>81</v>
       </c>
@@ -4512,7 +4329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="1">
         <v>68</v>
       </c>
@@ -4529,7 +4346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="1">
         <v>61</v>
       </c>
@@ -4546,7 +4363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="1">
         <v>8</v>
       </c>
@@ -4563,7 +4380,7 @@
         <v>0.96532594936184646</v>
       </c>
     </row>
-    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="1">
         <v>331</v>
       </c>
@@ -4580,7 +4397,7 @@
         <v>1.646245164624516E-3</v>
       </c>
     </row>
-    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="1">
         <v>332</v>
       </c>
@@ -4937,7 +4754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="1">
         <v>370</v>
       </c>
@@ -4954,7 +4771,7 @@
         <v>0.134621057292997</v>
       </c>
     </row>
-    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="1">
         <v>120</v>
       </c>
@@ -4971,7 +4788,7 @@
         <v>3.5757709964379873E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="1">
         <v>366</v>
       </c>
@@ -4988,7 +4805,7 @@
         <v>2.3214134465745669E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="1">
         <v>27</v>
       </c>
@@ -5005,7 +4822,7 @@
         <v>3.2958433086669972E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="1">
         <v>31</v>
       </c>
@@ -5022,7 +4839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="1">
         <v>58</v>
       </c>
@@ -5039,7 +4856,7 @@
         <v>0.79815484937119208</v>
       </c>
     </row>
-    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="1">
         <v>109</v>
       </c>
@@ -5056,7 +4873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="1">
         <v>333</v>
       </c>
@@ -5073,7 +4890,7 @@
         <v>3.841564384156438E-3</v>
       </c>
     </row>
-    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="1">
         <v>125</v>
       </c>
@@ -5090,7 +4907,7 @@
         <v>0.1579465383968629</v>
       </c>
     </row>
-    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="1">
         <v>365</v>
       </c>
@@ -5107,7 +4924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="1">
         <v>101</v>
       </c>
@@ -5124,7 +4941,7 @@
         <v>0.64918826781227201</v>
       </c>
     </row>
-    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="1">
         <v>46</v>
       </c>
@@ -5141,7 +4958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="1">
         <v>116</v>
       </c>
@@ -5158,7 +4975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="1">
         <v>336</v>
       </c>
@@ -5175,7 +4992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="1">
         <v>100</v>
       </c>
@@ -5192,7 +5009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="1">
         <v>337</v>
       </c>
@@ -5209,7 +5026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="1">
         <v>42</v>
       </c>
@@ -5226,7 +5043,7 @@
         <v>0.22391410311406079</v>
       </c>
     </row>
-    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="1">
         <v>76</v>
       </c>
@@ -5243,7 +5060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="1">
         <v>105</v>
       </c>
@@ -5260,7 +5077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="1">
         <v>334</v>
       </c>
@@ -5277,7 +5094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="1">
         <v>86</v>
       </c>
@@ -5294,7 +5111,7 @@
         <v>0.28126925061650448</v>
       </c>
     </row>
-    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="1">
         <v>335</v>
       </c>
@@ -5311,7 +5128,7 @@
         <v>1.2407619935443639E-2</v>
       </c>
     </row>
-    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="1">
         <v>24</v>
       </c>
@@ -5328,7 +5145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="1">
         <v>362</v>
       </c>
@@ -5345,7 +5162,7 @@
         <v>6.839000683900068E-5</v>
       </c>
     </row>
-    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="1">
         <v>29</v>
       </c>
@@ -5362,7 +5179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="1">
         <v>80</v>
       </c>
@@ -5379,7 +5196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="1">
         <v>338</v>
       </c>
@@ -5396,7 +5213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="1">
         <v>138</v>
       </c>
@@ -5413,7 +5230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="1">
         <v>140</v>
       </c>
@@ -5447,7 +5264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="1">
         <v>141</v>
       </c>
@@ -5787,7 +5604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224" s="1">
         <v>359</v>
       </c>
@@ -5804,7 +5621,7 @@
         <v>0.48166548561682748</v>
       </c>
     </row>
-    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A225" s="1">
         <v>340</v>
       </c>
@@ -5821,7 +5638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A226" s="1">
         <v>22</v>
       </c>
@@ -5838,7 +5655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A227" s="1">
         <v>96</v>
       </c>
@@ -5855,7 +5672,7 @@
         <v>0.70275640100091408</v>
       </c>
     </row>
-    <row r="228" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A228" s="1">
         <v>33</v>
       </c>
@@ -5872,7 +5689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A229" s="1">
         <v>117</v>
       </c>
@@ -5889,7 +5706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A230" s="1">
         <v>339</v>
       </c>
@@ -5906,7 +5723,7 @@
         <v>2.341490451249045E-2</v>
       </c>
     </row>
-    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A231" s="1">
         <v>70</v>
       </c>
@@ -5923,7 +5740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="1">
         <v>60</v>
       </c>
@@ -5940,7 +5757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="1">
         <v>66</v>
       </c>
@@ -5957,7 +5774,7 @@
         <v>0.25032567776301018</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="1">
         <v>39</v>
       </c>
@@ -5974,7 +5791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="1">
         <v>78</v>
       </c>
@@ -5991,7 +5808,7 @@
         <v>0.12715879875518479</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="1">
         <v>341</v>
       </c>
@@ -6008,7 +5825,7 @@
         <v>0.11353338766233879</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="1">
         <v>21</v>
       </c>
@@ -6025,7 +5842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="1">
         <v>114</v>
       </c>
@@ -6042,7 +5859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="1">
         <v>342</v>
       </c>
@@ -6059,7 +5876,7 @@
         <v>5.4642443064244301E-3</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="1">
         <v>63</v>
       </c>
@@ -6076,7 +5893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="1">
         <v>119</v>
       </c>
@@ -6093,7 +5910,7 @@
         <v>0.79429731808736814</v>
       </c>
     </row>
-    <row r="242" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="1">
         <v>343</v>
       </c>
@@ -6110,7 +5927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="1">
         <v>136</v>
       </c>
@@ -6467,7 +6284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="1">
         <v>360</v>
       </c>
@@ -6484,7 +6301,7 @@
         <v>0.17091135363853979</v>
       </c>
     </row>
-    <row r="265" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="1">
         <v>47</v>
       </c>
@@ -6501,7 +6318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="1">
         <v>44</v>
       </c>
@@ -6518,7 +6335,7 @@
         <v>0.32382763521744129</v>
       </c>
     </row>
-    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="1">
         <v>55</v>
       </c>
@@ -6535,7 +6352,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="1">
         <v>77</v>
       </c>
@@ -6552,7 +6369,7 @@
         <v>0.45543761613824829</v>
       </c>
     </row>
-    <row r="269" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="1">
         <v>344</v>
       </c>
@@ -6569,7 +6386,7 @@
         <v>8.8096098809609877E-3</v>
       </c>
     </row>
-    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="1">
         <v>89</v>
       </c>
@@ -6586,7 +6403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="1">
         <v>36</v>
       </c>
@@ -6603,7 +6420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="1">
         <v>4</v>
       </c>
@@ -6620,7 +6437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="273" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="1">
         <v>346</v>
       </c>
@@ -6637,7 +6454,7 @@
         <v>3.9959303995930389E-4</v>
       </c>
     </row>
-    <row r="274" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="1">
         <v>7</v>
       </c>
@@ -6654,7 +6471,7 @@
         <v>0.39480136465031063</v>
       </c>
     </row>
-    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="1">
         <v>145</v>
       </c>
@@ -6671,7 +6488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="1">
         <v>143</v>
       </c>
@@ -6688,7 +6505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="1">
         <v>71</v>
       </c>
@@ -6705,7 +6522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="1">
         <v>13</v>
       </c>
@@ -6722,7 +6539,7 @@
         <v>0.23549314237581301</v>
       </c>
     </row>
-    <row r="279" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="1">
         <v>94</v>
       </c>
@@ -6756,7 +6573,7 @@
         <v>0.14598219642993759</v>
       </c>
     </row>
-    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="1">
         <v>72</v>
       </c>
@@ -6773,7 +6590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="1">
         <v>83</v>
       </c>
@@ -7113,7 +6930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="1">
         <v>345</v>
       </c>
@@ -7130,7 +6947,7 @@
         <v>0.62376244531994651</v>
       </c>
     </row>
-    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="1">
         <v>124</v>
       </c>
@@ -7147,7 +6964,7 @@
         <v>6.0872298986459931E-3</v>
       </c>
     </row>
-    <row r="304" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="1">
         <v>357</v>
       </c>
@@ -7164,7 +6981,7 @@
         <v>0.12422935438275989</v>
       </c>
     </row>
-    <row r="305" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="1">
         <v>51</v>
       </c>
@@ -7181,7 +6998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="1">
         <v>98</v>
       </c>
@@ -7198,7 +7015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="1">
         <v>348</v>
       </c>
@@ -7215,7 +7032,7 @@
         <v>5.2113185211318518E-6</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="1">
         <v>6</v>
       </c>
@@ -7232,7 +7049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="1">
         <v>34</v>
       </c>
@@ -7249,7 +7066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="1">
         <v>37</v>
       </c>
@@ -7266,7 +7083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="1">
         <v>69</v>
       </c>
@@ -7283,7 +7100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="1">
         <v>347</v>
       </c>
@@ -7300,7 +7117,7 @@
         <v>6.5166883516688337E-5</v>
       </c>
     </row>
-    <row r="313" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="1">
         <v>85</v>
       </c>
@@ -7317,7 +7134,7 @@
         <v>0.83886768607262796</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="1">
         <v>350</v>
       </c>
@@ -7334,7 +7151,7 @@
         <v>1.856300185630018E-3</v>
       </c>
     </row>
-    <row r="315" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="1">
         <v>23</v>
       </c>
@@ -7351,7 +7168,7 @@
         <v>0.93374693709011558</v>
       </c>
     </row>
-    <row r="316" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="1">
         <v>56</v>
       </c>
@@ -7368,7 +7185,7 @@
         <v>0.52404713606528763</v>
       </c>
     </row>
-    <row r="317" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="1">
         <v>111</v>
       </c>
@@ -7385,7 +7202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="1">
         <v>351</v>
       </c>
@@ -7742,7 +7559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A339" s="1">
         <v>358</v>
       </c>
@@ -7759,7 +7576,7 @@
         <v>2.8787565964615281E-2</v>
       </c>
     </row>
-    <row r="340" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A340" s="1">
         <v>67</v>
       </c>
@@ -7776,7 +7593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="341" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A341" s="1">
         <v>103</v>
       </c>
@@ -7793,7 +7610,7 @@
         <v>1.198339642314117E-2</v>
       </c>
     </row>
-    <row r="342" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A342" s="1">
         <v>75</v>
       </c>
@@ -7810,7 +7627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A343" s="1">
         <v>49</v>
       </c>
@@ -7827,7 +7644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="344" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A344" s="1">
         <v>97</v>
       </c>
@@ -7844,7 +7661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="345" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A345" s="1">
         <v>353</v>
       </c>
@@ -7861,7 +7678,7 @@
         <v>1.9067133906713388E-2</v>
       </c>
     </row>
-    <row r="346" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A346" s="1">
         <v>74</v>
       </c>
@@ -7878,7 +7695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="347" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A347" s="1">
         <v>41</v>
       </c>
@@ -7895,7 +7712,7 @@
         <v>0.22793297675270141</v>
       </c>
     </row>
-    <row r="348" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A348" s="1">
         <v>14</v>
       </c>
@@ -7912,7 +7729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="349" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A349" s="1">
         <v>115</v>
       </c>
@@ -7929,7 +7746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="350" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A350" s="1">
         <v>352</v>
       </c>
@@ -7946,7 +7763,7 @@
         <v>3.2081314512131448E-2</v>
       </c>
     </row>
-    <row r="351" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A351" s="1">
         <v>142</v>
       </c>
@@ -8303,7 +8120,7 @@
         <v>5.1097105109710508E-2</v>
       </c>
     </row>
-    <row r="372" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A372" s="1">
         <v>355</v>
       </c>

</xml_diff>